<commit_message>
Updating Error List file 12-8-25
</commit_message>
<xml_diff>
--- a/Error Inventory/API Error Consolidated List.xlsx
+++ b/Error Inventory/API Error Consolidated List.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\eagnmnwbp130a.usa.dce.usps.gov\VDIProfiles$\fsbtg0\Documents\API Consolidated file to upload\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{221AFA77-C70C-4A96-B5FD-8FDE26F499FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F549680-687E-456D-A4F1-C57345E92A81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="13920" firstSheet="11" activeTab="12" xr2:uid="{BD4CA92B-BD2B-408A-B66B-5389FE5197CE}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="13785" firstSheet="3" activeTab="4" xr2:uid="{BD4CA92B-BD2B-408A-B66B-5389FE5197CE}"/>
   </bookViews>
   <sheets>
     <sheet name="General Errors" sheetId="9" r:id="rId1"/>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4010" uniqueCount="1009">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4050" uniqueCount="1014">
   <si>
     <t>API</t>
   </si>
@@ -3118,6 +3118,21 @@
   </si>
   <si>
     <t>barcode&lt;barcode &gt;has manifested and is not eligible to be added to a SCAN Form</t>
+  </si>
+  <si>
+    <t>imageInfo.imageType, imageInfo.labelType</t>
+  </si>
+  <si>
+    <t>&lt;labelType&gt; currently does not support imageInfo.imageType of &lt;imageType&gt;</t>
+  </si>
+  <si>
+    <t>EPL format does not same page or separate page receipt functionality.</t>
+  </si>
+  <si>
+    <t>brandingImageFormat currently does not support imageInfo.imageType of 'EPL203DPI' or 'EPL300DPI'</t>
+  </si>
+  <si>
+    <t>label with trackingNumber '%s' is not eligible for containerization</t>
   </si>
 </sst>
 </file>
@@ -3261,7 +3276,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -3398,6 +3413,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Accent1" xfId="1" builtinId="29"/>
@@ -7649,7 +7667,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
@@ -8029,6 +8047,29 @@
         <v>681</v>
       </c>
     </row>
+    <row r="17" spans="1:7">
+      <c r="A17" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="B17" s="10">
+        <v>400</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D17" s="10" t="s">
+        <v>957</v>
+      </c>
+      <c r="E17" s="17">
+        <v>160402</v>
+      </c>
+      <c r="F17" s="17" t="s">
+        <v>754</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>1013</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -8039,7 +8080,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:G232"/>
+  <dimension ref="A1:G235"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.140625" bestFit="1" customWidth="1"/>
@@ -13377,6 +13418,75 @@
         <v>1002</v>
       </c>
     </row>
+    <row r="233" spans="1:7">
+      <c r="A233" s="20" t="s">
+        <v>87</v>
+      </c>
+      <c r="B233" s="20">
+        <v>400</v>
+      </c>
+      <c r="C233" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="D233" s="21" t="s">
+        <v>959</v>
+      </c>
+      <c r="E233" s="17">
+        <v>160399</v>
+      </c>
+      <c r="F233" s="17" t="s">
+        <v>1009</v>
+      </c>
+      <c r="G233" s="48" t="s">
+        <v>1010</v>
+      </c>
+    </row>
+    <row r="234" spans="1:7" ht="30">
+      <c r="A234" s="20" t="s">
+        <v>87</v>
+      </c>
+      <c r="B234" s="20">
+        <v>400</v>
+      </c>
+      <c r="C234" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="D234" s="21" t="s">
+        <v>959</v>
+      </c>
+      <c r="E234" s="17">
+        <v>160400</v>
+      </c>
+      <c r="F234" s="37" t="s">
+        <v>694</v>
+      </c>
+      <c r="G234" s="48" t="s">
+        <v>1011</v>
+      </c>
+    </row>
+    <row r="235" spans="1:7">
+      <c r="A235" s="20" t="s">
+        <v>87</v>
+      </c>
+      <c r="B235" s="20">
+        <v>400</v>
+      </c>
+      <c r="C235" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="D235" s="21" t="s">
+        <v>959</v>
+      </c>
+      <c r="E235" s="17">
+        <v>160401</v>
+      </c>
+      <c r="F235" s="37" t="s">
+        <v>841</v>
+      </c>
+      <c r="G235" s="2" t="s">
+        <v>1012</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G1" xr:uid="{A36F69E6-5AC8-443F-8567-4E3FB7E927F1}"/>
   <phoneticPr fontId="9" type="noConversion"/>
@@ -13390,7 +13500,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:G191"/>
+  <dimension ref="A1:G193"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="23" bestFit="1" customWidth="1"/>
@@ -17752,6 +17862,52 @@
       </c>
       <c r="G191" s="2" t="s">
         <v>1002</v>
+      </c>
+    </row>
+    <row r="192" spans="1:7" ht="30">
+      <c r="A192" s="10" t="s">
+        <v>369</v>
+      </c>
+      <c r="B192" s="21">
+        <v>400</v>
+      </c>
+      <c r="C192" s="21" t="s">
+        <v>18</v>
+      </c>
+      <c r="D192" s="10" t="s">
+        <v>965</v>
+      </c>
+      <c r="E192" s="17">
+        <v>160400</v>
+      </c>
+      <c r="F192" s="33" t="s">
+        <v>694</v>
+      </c>
+      <c r="G192" s="48" t="s">
+        <v>1011</v>
+      </c>
+    </row>
+    <row r="193" spans="1:7">
+      <c r="A193" s="10" t="s">
+        <v>369</v>
+      </c>
+      <c r="B193" s="21">
+        <v>400</v>
+      </c>
+      <c r="C193" s="21" t="s">
+        <v>18</v>
+      </c>
+      <c r="D193" s="10" t="s">
+        <v>965</v>
+      </c>
+      <c r="E193" s="17">
+        <v>160401</v>
+      </c>
+      <c r="F193" s="33" t="s">
+        <v>841</v>
+      </c>
+      <c r="G193" s="2" t="s">
+        <v>1012</v>
       </c>
     </row>
   </sheetData>
@@ -18667,7 +18823,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
@@ -19520,6 +19676,52 @@
       </c>
       <c r="G37" s="2" t="s">
         <v>1002</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" ht="30">
+      <c r="A38" t="s">
+        <v>475</v>
+      </c>
+      <c r="B38">
+        <v>400</v>
+      </c>
+      <c r="C38" t="s">
+        <v>18</v>
+      </c>
+      <c r="D38" t="s">
+        <v>970</v>
+      </c>
+      <c r="E38" s="26">
+        <v>160400</v>
+      </c>
+      <c r="F38" s="33" t="s">
+        <v>694</v>
+      </c>
+      <c r="G38" s="48" t="s">
+        <v>1011</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7">
+      <c r="A39" t="s">
+        <v>475</v>
+      </c>
+      <c r="B39">
+        <v>400</v>
+      </c>
+      <c r="C39" t="s">
+        <v>18</v>
+      </c>
+      <c r="D39" t="s">
+        <v>970</v>
+      </c>
+      <c r="E39" s="26">
+        <v>160401</v>
+      </c>
+      <c r="F39" s="33" t="s">
+        <v>841</v>
+      </c>
+      <c r="G39" s="2" t="s">
+        <v>1012</v>
       </c>
     </row>
   </sheetData>
@@ -20233,6 +20435,19 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <TaxCatchAll xmlns="9cf85ca5-4acf-45da-adaa-d6bfc34b6c9f" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2595f96f-d2aa-4fa4-b5ed-10baae53ecb9">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100BD1EFD7F07544F4C8A5DF6ACE5557D0F" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="0a46465e297c47d8b88a71685f887e65">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="2595f96f-d2aa-4fa4-b5ed-10baae53ecb9" xmlns:ns3="9cf85ca5-4acf-45da-adaa-d6bfc34b6c9f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4503a5f252426d71f93d44927b16e869" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -20478,19 +20693,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <TaxCatchAll xmlns="9cf85ca5-4acf-45da-adaa-d6bfc34b6c9f" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2595f96f-d2aa-4fa4-b5ed-10baae53ecb9">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D590CCA9-7961-4660-BBC6-10104A0DDFD4}">
   <ds:schemaRefs>
@@ -20500,6 +20702,24 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B3DC8D4E-C199-4BF9-AF5D-F16C7D7041E1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="2595f96f-d2aa-4fa4-b5ed-10baae53ecb9"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="9cf85ca5-4acf-45da-adaa-d6bfc34b6c9f"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F11AB0D6-FBA0-4F11-8778-05A9ADBB93A5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -20519,24 +20739,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B3DC8D4E-C199-4BF9-AF5D-F16C7D7041E1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="2595f96f-d2aa-4fa4-b5ed-10baae53ecb9"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="9cf85ca5-4acf-45da-adaa-d6bfc34b6c9f"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{6c9b68e5-0371-4f27-93af-8d15f794dc29}" enabled="1" method="Privileged" siteId="{a01f407a-85cb-4a16-98bb-f28e6384bd28}" removed="0"/>

</xml_diff>

<commit_message>
Updated Error List file for 3/25/2026 Release
</commit_message>
<xml_diff>
--- a/Error Inventory/API Error Consolidated List.xlsx
+++ b/Error Inventory/API Error Consolidated List.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\eagnmnwbp130a.usa.dce.usps.gov\VDIProfiles$\fsbtg0\Documents\API Consolidated file to upload\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usps365-my.sharepoint.com/personal/norman_negron-munoz_usps_gov/Documents/Documents/EMAS API/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F53487B-9017-4953-8EAD-F36B8AB737A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{EEC637CC-2ACF-49A4-B5A4-20E89772DFF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="13785" firstSheet="9" activeTab="10" xr2:uid="{BD4CA92B-BD2B-408A-B66B-5389FE5197CE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="13920" firstSheet="3" activeTab="4" xr2:uid="{BD4CA92B-BD2B-408A-B66B-5389FE5197CE}"/>
   </bookViews>
   <sheets>
     <sheet name="General Errors" sheetId="9" r:id="rId1"/>
@@ -34,7 +34,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Addresses!$A$1:$G$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Carrier Pickup'!$A$1:$G$73</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Domestic Labels Outbound'!$A$1:$G$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Domestic Prices'!$A$1:$G$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Domestic Prices'!$A$1:$G$48</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'General Errors'!$A$1:$D$82</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'International Prices'!$A$1:$G$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">Tracking!$A$1:$G$6</definedName>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4075" uniqueCount="1019">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4187" uniqueCount="1043">
   <si>
     <t>API</t>
   </si>
@@ -3148,6 +3148,78 @@
   </si>
   <si>
     <t>destinationEntryFacilityType must be 'DESTINATION_DELIVERY_UNIT' when processingCategory is 'MIXED'</t>
+  </si>
+  <si>
+    <t>imiType can only be IMI_STD unless imageInfo.labelType is IMI_DATA_ONLY</t>
+  </si>
+  <si>
+    <t>indiciaDescription</t>
+  </si>
+  <si>
+    <t>indiciaID not found</t>
+  </si>
+  <si>
+    <t>indiciaID</t>
+  </si>
+  <si>
+    <t>030025</t>
+  </si>
+  <si>
+    <t>030026</t>
+  </si>
+  <si>
+    <t>030027</t>
+  </si>
+  <si>
+    <t>030028</t>
+  </si>
+  <si>
+    <t>030029</t>
+  </si>
+  <si>
+    <t>030030</t>
+  </si>
+  <si>
+    <t>030031</t>
+  </si>
+  <si>
+    <t>030032</t>
+  </si>
+  <si>
+    <t>030033</t>
+  </si>
+  <si>
+    <t>A minimum item value greater than 500 is required for this extra service.</t>
+  </si>
+  <si>
+    <t>Provided weight exceeds maximum allowed for First Class Postcards.</t>
+  </si>
+  <si>
+    <t>Provided dimensions do not meet minimum allowed for First Class Postcards.</t>
+  </si>
+  <si>
+    <t>Provided dimensions exceed maximum allowed for First Class Postcards.</t>
+  </si>
+  <si>
+    <t>You must have a valid province code when requesting Delivery Duties pricing for %.</t>
+  </si>
+  <si>
+    <t>One or more extra services are not available for international pieces in this price group.  (Based on the mailClass, countryCode, and rateIndicator.)</t>
+  </si>
+  <si>
+    <t>DDP is not available for the provided country and product options.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The provided invoice date is not supported. The earliest supported date is </t>
+  </si>
+  <si>
+    <t>The provided API Agreement Type is not supported.</t>
+  </si>
+  <si>
+    <t>extraServiceCodes</t>
+  </si>
+  <si>
+    <t>date</t>
   </si>
 </sst>
 </file>
@@ -3291,7 +3363,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -3431,6 +3503,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Accent1" xfId="1" builtinId="29"/>
@@ -8118,7 +8192,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:G235"/>
+  <dimension ref="A1:G237"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.140625" bestFit="1" customWidth="1"/>
@@ -13523,6 +13597,52 @@
       </c>
       <c r="G235" s="2" t="s">
         <v>1011</v>
+      </c>
+    </row>
+    <row r="236" spans="1:7">
+      <c r="A236" s="20" t="s">
+        <v>87</v>
+      </c>
+      <c r="B236" s="20">
+        <v>400</v>
+      </c>
+      <c r="C236" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="D236" s="50" t="s">
+        <v>1003</v>
+      </c>
+      <c r="E236" s="17">
+        <v>160408</v>
+      </c>
+      <c r="F236" s="17" t="s">
+        <v>1020</v>
+      </c>
+      <c r="G236" s="49" t="s">
+        <v>1019</v>
+      </c>
+    </row>
+    <row r="237" spans="1:7">
+      <c r="A237" s="20" t="s">
+        <v>87</v>
+      </c>
+      <c r="B237" s="20">
+        <v>400</v>
+      </c>
+      <c r="C237" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="D237" s="50" t="s">
+        <v>1003</v>
+      </c>
+      <c r="E237" s="17">
+        <v>160409</v>
+      </c>
+      <c r="F237" s="17" t="s">
+        <v>1022</v>
+      </c>
+      <c r="G237" s="49" t="s">
+        <v>1021</v>
       </c>
     </row>
   </sheetData>
@@ -17959,7 +18079,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G48"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.5703125" style="10" bestFit="1" customWidth="1"/>
@@ -18573,7 +18693,7 @@
         <v>668</v>
       </c>
     </row>
-    <row r="28" spans="1:7">
+    <row r="28" spans="1:7" ht="30">
       <c r="A28" s="10" t="s">
         <v>415</v>
       </c>
@@ -18583,20 +18703,20 @@
       <c r="C28" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="D28" s="10" t="s">
-        <v>968</v>
+      <c r="D28" s="11" t="s">
+        <v>966</v>
       </c>
       <c r="E28" s="24" t="s">
-        <v>468</v>
+        <v>1023</v>
       </c>
       <c r="F28" s="33" t="s">
-        <v>804</v>
-      </c>
-      <c r="G28" s="11" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7">
+        <v>810</v>
+      </c>
+      <c r="G28" s="10" t="s">
+        <v>1032</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="30">
       <c r="A29" s="10" t="s">
         <v>415</v>
       </c>
@@ -18606,20 +18726,20 @@
       <c r="C29" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="D29" s="10" t="s">
-        <v>968</v>
+      <c r="D29" s="11" t="s">
+        <v>966</v>
       </c>
       <c r="E29" s="24" t="s">
-        <v>469</v>
+        <v>1024</v>
       </c>
       <c r="F29" s="33" t="s">
-        <v>805</v>
-      </c>
-      <c r="G29" s="11" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7">
+        <v>764</v>
+      </c>
+      <c r="G29" s="10" t="s">
+        <v>1033</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="30">
       <c r="A30" s="10" t="s">
         <v>415</v>
       </c>
@@ -18629,20 +18749,20 @@
       <c r="C30" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="D30" s="17" t="s">
-        <v>968</v>
-      </c>
-      <c r="E30" s="33" t="s">
-        <v>430</v>
+      <c r="D30" s="11" t="s">
+        <v>966</v>
+      </c>
+      <c r="E30" s="24" t="s">
+        <v>1025</v>
       </c>
       <c r="F30" s="33" t="s">
         <v>801</v>
       </c>
       <c r="G30" s="10" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7">
+        <v>1034</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="30">
       <c r="A31" s="10" t="s">
         <v>415</v>
       </c>
@@ -18652,20 +18772,20 @@
       <c r="C31" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="D31" s="17" t="s">
-        <v>968</v>
-      </c>
-      <c r="E31" s="33" t="s">
-        <v>431</v>
-      </c>
-      <c r="F31" s="41" t="s">
-        <v>802</v>
+      <c r="D31" s="11" t="s">
+        <v>966</v>
+      </c>
+      <c r="E31" s="24" t="s">
+        <v>1026</v>
+      </c>
+      <c r="F31" s="33" t="s">
+        <v>801</v>
       </c>
       <c r="G31" s="10" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7">
+        <v>1035</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="30">
       <c r="A32" s="10" t="s">
         <v>415</v>
       </c>
@@ -18675,20 +18795,18 @@
       <c r="C32" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="D32" s="17" t="s">
-        <v>968</v>
-      </c>
-      <c r="E32" s="33" t="s">
-        <v>433</v>
-      </c>
-      <c r="F32" s="41" t="s">
-        <v>803</v>
-      </c>
+      <c r="D32" s="11" t="s">
+        <v>966</v>
+      </c>
+      <c r="E32" s="24" t="s">
+        <v>1027</v>
+      </c>
+      <c r="F32" s="33"/>
       <c r="G32" s="10" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7">
+        <v>1036</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" ht="30">
       <c r="A33" s="10" t="s">
         <v>415</v>
       </c>
@@ -18698,20 +18816,20 @@
       <c r="C33" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="D33" s="17" t="s">
-        <v>968</v>
+      <c r="D33" s="11" t="s">
+        <v>966</v>
       </c>
       <c r="E33" s="24" t="s">
-        <v>434</v>
-      </c>
-      <c r="F33" s="37" t="s">
-        <v>804</v>
+        <v>1028</v>
+      </c>
+      <c r="F33" s="33" t="s">
+        <v>1041</v>
       </c>
       <c r="G33" s="10" t="s">
-        <v>435</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7">
+        <v>1037</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" ht="30">
       <c r="A34" s="10" t="s">
         <v>415</v>
       </c>
@@ -18721,20 +18839,18 @@
       <c r="C34" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="D34" s="17" t="s">
-        <v>968</v>
+      <c r="D34" s="11" t="s">
+        <v>966</v>
       </c>
       <c r="E34" s="24" t="s">
-        <v>436</v>
-      </c>
-      <c r="F34" s="37" t="s">
-        <v>805</v>
-      </c>
+        <v>1029</v>
+      </c>
+      <c r="F34" s="33"/>
       <c r="G34" s="10" t="s">
-        <v>435</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7">
+        <v>1038</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" ht="30">
       <c r="A35" s="10" t="s">
         <v>415</v>
       </c>
@@ -18744,20 +18860,20 @@
       <c r="C35" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="D35" s="17" t="s">
-        <v>968</v>
+      <c r="D35" s="11" t="s">
+        <v>966</v>
       </c>
       <c r="E35" s="24" t="s">
-        <v>437</v>
-      </c>
-      <c r="F35" s="37" t="s">
-        <v>806</v>
+        <v>1030</v>
+      </c>
+      <c r="F35" s="33" t="s">
+        <v>1042</v>
       </c>
       <c r="G35" s="10" t="s">
-        <v>438</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7">
+        <v>1039</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="30">
       <c r="A36" s="10" t="s">
         <v>415</v>
       </c>
@@ -18767,20 +18883,18 @@
       <c r="C36" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="D36" s="17" t="s">
-        <v>968</v>
+      <c r="D36" s="11" t="s">
+        <v>966</v>
       </c>
       <c r="E36" s="24" t="s">
-        <v>439</v>
-      </c>
-      <c r="F36" s="37" t="s">
-        <v>807</v>
-      </c>
+        <v>1031</v>
+      </c>
+      <c r="F36" s="33"/>
       <c r="G36" s="10" t="s">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" ht="30">
+        <v>1040</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7">
       <c r="A37" s="10" t="s">
         <v>415</v>
       </c>
@@ -18793,17 +18907,17 @@
       <c r="D37" s="10" t="s">
         <v>968</v>
       </c>
-      <c r="E37" s="24">
-        <v>160289</v>
-      </c>
-      <c r="F37" s="2" t="s">
-        <v>808</v>
-      </c>
-      <c r="G37" s="22" t="s">
-        <v>665</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" ht="30">
+      <c r="E37" s="24" t="s">
+        <v>468</v>
+      </c>
+      <c r="F37" s="33" t="s">
+        <v>804</v>
+      </c>
+      <c r="G37" s="11" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7">
       <c r="A38" s="10" t="s">
         <v>415</v>
       </c>
@@ -18816,17 +18930,17 @@
       <c r="D38" s="10" t="s">
         <v>968</v>
       </c>
-      <c r="E38" s="24">
-        <v>160290</v>
-      </c>
-      <c r="F38" s="2" t="s">
-        <v>809</v>
-      </c>
-      <c r="G38" s="22" t="s">
-        <v>666</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" ht="30">
+      <c r="E38" s="24" t="s">
+        <v>469</v>
+      </c>
+      <c r="F38" s="33" t="s">
+        <v>805</v>
+      </c>
+      <c r="G38" s="11" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7">
       <c r="A39" s="10" t="s">
         <v>415</v>
       </c>
@@ -18836,21 +18950,228 @@
       <c r="C39" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="D39" s="10" t="s">
+      <c r="D39" s="17" t="s">
         <v>968</v>
       </c>
-      <c r="E39" s="24">
+      <c r="E39" s="33" t="s">
+        <v>430</v>
+      </c>
+      <c r="F39" s="33" t="s">
+        <v>801</v>
+      </c>
+      <c r="G39" s="10" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7">
+      <c r="A40" s="10" t="s">
+        <v>415</v>
+      </c>
+      <c r="B40" s="10">
+        <v>400</v>
+      </c>
+      <c r="C40" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D40" s="17" t="s">
+        <v>968</v>
+      </c>
+      <c r="E40" s="33" t="s">
+        <v>431</v>
+      </c>
+      <c r="F40" s="41" t="s">
+        <v>802</v>
+      </c>
+      <c r="G40" s="10" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7">
+      <c r="A41" s="10" t="s">
+        <v>415</v>
+      </c>
+      <c r="B41" s="10">
+        <v>400</v>
+      </c>
+      <c r="C41" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D41" s="17" t="s">
+        <v>968</v>
+      </c>
+      <c r="E41" s="33" t="s">
+        <v>433</v>
+      </c>
+      <c r="F41" s="41" t="s">
+        <v>803</v>
+      </c>
+      <c r="G41" s="10" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7">
+      <c r="A42" s="10" t="s">
+        <v>415</v>
+      </c>
+      <c r="B42" s="10">
+        <v>400</v>
+      </c>
+      <c r="C42" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D42" s="17" t="s">
+        <v>968</v>
+      </c>
+      <c r="E42" s="24" t="s">
+        <v>434</v>
+      </c>
+      <c r="F42" s="37" t="s">
+        <v>804</v>
+      </c>
+      <c r="G42" s="10" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7">
+      <c r="A43" s="10" t="s">
+        <v>415</v>
+      </c>
+      <c r="B43" s="10">
+        <v>400</v>
+      </c>
+      <c r="C43" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D43" s="17" t="s">
+        <v>968</v>
+      </c>
+      <c r="E43" s="24" t="s">
+        <v>436</v>
+      </c>
+      <c r="F43" s="37" t="s">
+        <v>805</v>
+      </c>
+      <c r="G43" s="10" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7">
+      <c r="A44" s="10" t="s">
+        <v>415</v>
+      </c>
+      <c r="B44" s="10">
+        <v>400</v>
+      </c>
+      <c r="C44" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D44" s="17" t="s">
+        <v>968</v>
+      </c>
+      <c r="E44" s="24" t="s">
+        <v>437</v>
+      </c>
+      <c r="F44" s="37" t="s">
+        <v>806</v>
+      </c>
+      <c r="G44" s="10" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7">
+      <c r="A45" s="10" t="s">
+        <v>415</v>
+      </c>
+      <c r="B45" s="10">
+        <v>400</v>
+      </c>
+      <c r="C45" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D45" s="17" t="s">
+        <v>968</v>
+      </c>
+      <c r="E45" s="24" t="s">
+        <v>439</v>
+      </c>
+      <c r="F45" s="37" t="s">
+        <v>807</v>
+      </c>
+      <c r="G45" s="10" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" ht="30">
+      <c r="A46" s="10" t="s">
+        <v>415</v>
+      </c>
+      <c r="B46" s="10">
+        <v>400</v>
+      </c>
+      <c r="C46" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D46" s="10" t="s">
+        <v>968</v>
+      </c>
+      <c r="E46" s="24">
+        <v>160289</v>
+      </c>
+      <c r="F46" s="2" t="s">
+        <v>808</v>
+      </c>
+      <c r="G46" s="22" t="s">
+        <v>665</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" ht="30">
+      <c r="A47" s="10" t="s">
+        <v>415</v>
+      </c>
+      <c r="B47" s="10">
+        <v>400</v>
+      </c>
+      <c r="C47" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D47" s="10" t="s">
+        <v>968</v>
+      </c>
+      <c r="E47" s="24">
+        <v>160290</v>
+      </c>
+      <c r="F47" s="2" t="s">
+        <v>809</v>
+      </c>
+      <c r="G47" s="22" t="s">
+        <v>666</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" ht="30">
+      <c r="A48" s="10" t="s">
+        <v>415</v>
+      </c>
+      <c r="B48" s="10">
+        <v>400</v>
+      </c>
+      <c r="C48" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D48" s="10" t="s">
+        <v>968</v>
+      </c>
+      <c r="E48" s="24">
         <v>160306</v>
       </c>
-      <c r="F39" s="37" t="s">
+      <c r="F48" s="37" t="s">
         <v>710</v>
       </c>
-      <c r="G39" s="2" t="s">
+      <c r="G48" s="2" t="s">
         <v>688</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G39" xr:uid="{E9D67488-3AD8-4C63-B43B-F8AB72C087A6}"/>
+  <autoFilter ref="A1:G48" xr:uid="{E9D67488-3AD8-4C63-B43B-F8AB72C087A6}"/>
   <phoneticPr fontId="9" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -19864,7 +20185,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="19.28515625" style="2" customWidth="1"/>
@@ -20273,7 +20594,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="19" spans="1:7" s="11" customFormat="1" ht="30">
+    <row r="19" spans="1:7" s="11" customFormat="1">
       <c r="A19" s="11" t="s">
         <v>521</v>
       </c>
@@ -20283,7 +20604,7 @@
       <c r="C19" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="D19" s="11" t="s">
+      <c r="D19" s="50" t="s">
         <v>970</v>
       </c>
       <c r="E19" s="24" t="s">
@@ -20296,7 +20617,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="60">
+    <row r="20" spans="1:7" ht="35.25" customHeight="1">
       <c r="A20" s="11" t="s">
         <v>521</v>
       </c>
@@ -20319,7 +20640,7 @@
         <v>668</v>
       </c>
     </row>
-    <row r="21" spans="1:7">
+    <row r="21" spans="1:7" ht="30">
       <c r="A21" s="11" t="s">
         <v>521</v>
       </c>
@@ -20329,17 +20650,17 @@
       <c r="C21" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="D21" t="s">
-        <v>972</v>
-      </c>
-      <c r="E21" s="33" t="s">
-        <v>430</v>
-      </c>
-      <c r="F21" s="40" t="s">
-        <v>801</v>
+      <c r="D21" s="11" t="s">
+        <v>970</v>
+      </c>
+      <c r="E21" s="24" t="s">
+        <v>1023</v>
+      </c>
+      <c r="F21" s="33" t="s">
+        <v>810</v>
       </c>
       <c r="G21" s="10" t="s">
-        <v>252</v>
+        <v>1032</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="30">
@@ -20353,16 +20674,16 @@
         <v>18</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>972</v>
-      </c>
-      <c r="E22" s="33" t="s">
-        <v>431</v>
-      </c>
-      <c r="F22" s="40" t="s">
-        <v>802</v>
+        <v>970</v>
+      </c>
+      <c r="E22" s="24" t="s">
+        <v>1024</v>
+      </c>
+      <c r="F22" s="33" t="s">
+        <v>764</v>
       </c>
       <c r="G22" s="10" t="s">
-        <v>432</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="30">
@@ -20376,16 +20697,16 @@
         <v>18</v>
       </c>
       <c r="D23" s="11" t="s">
-        <v>972</v>
-      </c>
-      <c r="E23" s="33" t="s">
-        <v>433</v>
-      </c>
-      <c r="F23" s="40" t="s">
-        <v>803</v>
+        <v>970</v>
+      </c>
+      <c r="E23" s="24" t="s">
+        <v>1025</v>
+      </c>
+      <c r="F23" s="33" t="s">
+        <v>801</v>
       </c>
       <c r="G23" s="10" t="s">
-        <v>432</v>
+        <v>1034</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="30">
@@ -20399,16 +20720,16 @@
         <v>18</v>
       </c>
       <c r="D24" s="11" t="s">
-        <v>972</v>
+        <v>970</v>
       </c>
       <c r="E24" s="24" t="s">
-        <v>434</v>
-      </c>
-      <c r="F24" s="17" t="s">
-        <v>804</v>
+        <v>1026</v>
+      </c>
+      <c r="F24" s="33" t="s">
+        <v>801</v>
       </c>
       <c r="G24" s="10" t="s">
-        <v>435</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="30">
@@ -20422,16 +20743,14 @@
         <v>18</v>
       </c>
       <c r="D25" s="11" t="s">
-        <v>972</v>
+        <v>970</v>
       </c>
       <c r="E25" s="24" t="s">
-        <v>436</v>
-      </c>
-      <c r="F25" s="17" t="s">
-        <v>805</v>
-      </c>
+        <v>1027</v>
+      </c>
+      <c r="F25" s="33"/>
       <c r="G25" s="10" t="s">
-        <v>435</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="30">
@@ -20445,16 +20764,16 @@
         <v>18</v>
       </c>
       <c r="D26" s="11" t="s">
-        <v>972</v>
+        <v>970</v>
       </c>
       <c r="E26" s="24" t="s">
-        <v>437</v>
-      </c>
-      <c r="F26" s="17" t="s">
-        <v>806</v>
+        <v>1028</v>
+      </c>
+      <c r="F26" s="33" t="s">
+        <v>1041</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>438</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="30">
@@ -20468,16 +20787,14 @@
         <v>18</v>
       </c>
       <c r="D27" s="11" t="s">
-        <v>972</v>
+        <v>970</v>
       </c>
       <c r="E27" s="24" t="s">
-        <v>439</v>
-      </c>
-      <c r="F27" s="17" t="s">
-        <v>807</v>
-      </c>
+        <v>1029</v>
+      </c>
+      <c r="F27" s="33"/>
       <c r="G27" s="10" t="s">
-        <v>350</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="30">
@@ -20491,16 +20808,16 @@
         <v>18</v>
       </c>
       <c r="D28" s="11" t="s">
-        <v>972</v>
-      </c>
-      <c r="E28" s="24">
-        <v>160289</v>
-      </c>
-      <c r="F28" s="37" t="s">
-        <v>808</v>
+        <v>970</v>
+      </c>
+      <c r="E28" s="24" t="s">
+        <v>1030</v>
+      </c>
+      <c r="F28" s="33" t="s">
+        <v>1042</v>
       </c>
       <c r="G28" s="10" t="s">
-        <v>665</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="30">
@@ -20514,19 +20831,17 @@
         <v>18</v>
       </c>
       <c r="D29" s="11" t="s">
-        <v>972</v>
-      </c>
-      <c r="E29" s="24">
-        <v>160290</v>
-      </c>
-      <c r="F29" s="37" t="s">
-        <v>809</v>
-      </c>
+        <v>970</v>
+      </c>
+      <c r="E29" s="24" t="s">
+        <v>1031</v>
+      </c>
+      <c r="F29" s="33"/>
       <c r="G29" s="10" t="s">
-        <v>666</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" ht="30">
+        <v>1040</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7">
       <c r="A30" s="11" t="s">
         <v>521</v>
       </c>
@@ -20536,16 +20851,223 @@
       <c r="C30" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="D30" s="11" t="s">
+      <c r="D30" t="s">
         <v>972</v>
       </c>
-      <c r="E30" s="24">
+      <c r="E30" s="33" t="s">
+        <v>430</v>
+      </c>
+      <c r="F30" s="40" t="s">
+        <v>801</v>
+      </c>
+      <c r="G30" s="10" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="30">
+      <c r="A31" s="11" t="s">
+        <v>521</v>
+      </c>
+      <c r="B31" s="11">
+        <v>400</v>
+      </c>
+      <c r="C31" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D31" s="11" t="s">
+        <v>972</v>
+      </c>
+      <c r="E31" s="33" t="s">
+        <v>431</v>
+      </c>
+      <c r="F31" s="40" t="s">
+        <v>802</v>
+      </c>
+      <c r="G31" s="10" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="30">
+      <c r="A32" s="11" t="s">
+        <v>521</v>
+      </c>
+      <c r="B32" s="11">
+        <v>400</v>
+      </c>
+      <c r="C32" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D32" s="11" t="s">
+        <v>972</v>
+      </c>
+      <c r="E32" s="33" t="s">
+        <v>433</v>
+      </c>
+      <c r="F32" s="40" t="s">
+        <v>803</v>
+      </c>
+      <c r="G32" s="10" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" ht="30">
+      <c r="A33" s="11" t="s">
+        <v>521</v>
+      </c>
+      <c r="B33" s="11">
+        <v>400</v>
+      </c>
+      <c r="C33" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D33" s="11" t="s">
+        <v>972</v>
+      </c>
+      <c r="E33" s="24" t="s">
+        <v>434</v>
+      </c>
+      <c r="F33" s="17" t="s">
+        <v>804</v>
+      </c>
+      <c r="G33" s="10" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" ht="30">
+      <c r="A34" s="11" t="s">
+        <v>521</v>
+      </c>
+      <c r="B34" s="11">
+        <v>400</v>
+      </c>
+      <c r="C34" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D34" s="11" t="s">
+        <v>972</v>
+      </c>
+      <c r="E34" s="24" t="s">
+        <v>436</v>
+      </c>
+      <c r="F34" s="17" t="s">
+        <v>805</v>
+      </c>
+      <c r="G34" s="10" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" ht="30">
+      <c r="A35" s="11" t="s">
+        <v>521</v>
+      </c>
+      <c r="B35" s="11">
+        <v>400</v>
+      </c>
+      <c r="C35" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D35" s="11" t="s">
+        <v>972</v>
+      </c>
+      <c r="E35" s="24" t="s">
+        <v>437</v>
+      </c>
+      <c r="F35" s="17" t="s">
+        <v>806</v>
+      </c>
+      <c r="G35" s="10" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="30">
+      <c r="A36" s="11" t="s">
+        <v>521</v>
+      </c>
+      <c r="B36" s="11">
+        <v>400</v>
+      </c>
+      <c r="C36" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D36" s="11" t="s">
+        <v>972</v>
+      </c>
+      <c r="E36" s="24" t="s">
+        <v>439</v>
+      </c>
+      <c r="F36" s="17" t="s">
+        <v>807</v>
+      </c>
+      <c r="G36" s="10" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="30">
+      <c r="A37" s="11" t="s">
+        <v>521</v>
+      </c>
+      <c r="B37" s="11">
+        <v>400</v>
+      </c>
+      <c r="C37" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D37" s="11" t="s">
+        <v>972</v>
+      </c>
+      <c r="E37" s="24">
+        <v>160289</v>
+      </c>
+      <c r="F37" s="37" t="s">
+        <v>808</v>
+      </c>
+      <c r="G37" s="10" t="s">
+        <v>665</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" ht="30">
+      <c r="A38" s="11" t="s">
+        <v>521</v>
+      </c>
+      <c r="B38" s="11">
+        <v>400</v>
+      </c>
+      <c r="C38" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D38" s="11" t="s">
+        <v>972</v>
+      </c>
+      <c r="E38" s="24">
+        <v>160290</v>
+      </c>
+      <c r="F38" s="37" t="s">
+        <v>809</v>
+      </c>
+      <c r="G38" s="10" t="s">
+        <v>666</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" ht="30">
+      <c r="A39" s="11" t="s">
+        <v>521</v>
+      </c>
+      <c r="B39" s="11">
+        <v>400</v>
+      </c>
+      <c r="C39" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D39" s="11" t="s">
+        <v>972</v>
+      </c>
+      <c r="E39" s="24">
         <v>160396</v>
       </c>
-      <c r="F30" s="17" t="s">
+      <c r="F39" s="17" t="s">
         <v>1004</v>
       </c>
-      <c r="G30" s="2" t="s">
+      <c r="G39" s="2" t="s">
         <v>1005</v>
       </c>
     </row>
@@ -20556,6 +21078,19 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <TaxCatchAll xmlns="9cf85ca5-4acf-45da-adaa-d6bfc34b6c9f" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2595f96f-d2aa-4fa4-b5ed-10baae53ecb9">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100BD1EFD7F07544F4C8A5DF6ACE5557D0F" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="0a46465e297c47d8b88a71685f887e65">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="2595f96f-d2aa-4fa4-b5ed-10baae53ecb9" xmlns:ns3="9cf85ca5-4acf-45da-adaa-d6bfc34b6c9f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4503a5f252426d71f93d44927b16e869" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -20801,19 +21336,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <TaxCatchAll xmlns="9cf85ca5-4acf-45da-adaa-d6bfc34b6c9f" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2595f96f-d2aa-4fa4-b5ed-10baae53ecb9">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -20824,6 +21346,24 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B3DC8D4E-C199-4BF9-AF5D-F16C7D7041E1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="2595f96f-d2aa-4fa4-b5ed-10baae53ecb9"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="9cf85ca5-4acf-45da-adaa-d6bfc34b6c9f"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F11AB0D6-FBA0-4F11-8778-05A9ADBB93A5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -20843,24 +21383,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B3DC8D4E-C199-4BF9-AF5D-F16C7D7041E1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="2595f96f-d2aa-4fa4-b5ed-10baae53ecb9"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="9cf85ca5-4acf-45da-adaa-d6bfc34b6c9f"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D590CCA9-7961-4660-BBC6-10104A0DDFD4}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
API Error list update 4/30/2026
</commit_message>
<xml_diff>
--- a/Error Inventory/API Error Consolidated List.xlsx
+++ b/Error Inventory/API Error Consolidated List.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usps365-my.sharepoint.com/personal/norman_negron-munoz_usps_gov/Documents/Documents/EMAS API/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\eagnmnwbp130a.usa.dce.usps.gov\VDIProfiles$\fsbtg0\Documents\API Consolidated file to upload\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EEC637CC-2ACF-49A4-B5A4-20E89772DFF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A03FF57B-47E3-4436-9AB2-1F81EE5C8058}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="13920" firstSheet="3" activeTab="4" xr2:uid="{BD4CA92B-BD2B-408A-B66B-5389FE5197CE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="13920" activeTab="4" xr2:uid="{BD4CA92B-BD2B-408A-B66B-5389FE5197CE}"/>
   </bookViews>
   <sheets>
     <sheet name="General Errors" sheetId="9" r:id="rId1"/>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4187" uniqueCount="1043">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4235" uniqueCount="1045">
   <si>
     <t>API</t>
   </si>
@@ -3220,6 +3220,12 @@
   </si>
   <si>
     <t>date</t>
+  </si>
+  <si>
+    <t>Default address: The address you entered was found but more information is needed (such as an apartment, suite, or box number) to match to a specific address.</t>
+  </si>
+  <si>
+    <t>010007</t>
   </si>
 </sst>
 </file>
@@ -3363,7 +3369,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -3504,7 +3510,6 @@
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Accent1" xfId="1" builtinId="29"/>
@@ -7244,12 +7249,28 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:7">
-      <c r="A8" s="6"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="6"/>
-      <c r="F8" s="6"/>
-      <c r="G8" s="5"/>
+    <row r="8" spans="1:7" ht="75">
+      <c r="A8" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" s="19">
+        <v>400</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>954</v>
+      </c>
+      <c r="E8" s="27" t="s">
+        <v>1044</v>
+      </c>
+      <c r="F8" s="27" t="s">
+        <v>858</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>1043</v>
+      </c>
     </row>
     <row r="9" spans="1:7">
       <c r="B9" s="7"/>
@@ -8192,7 +8213,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:G237"/>
+  <dimension ref="A1:G244"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.140625" bestFit="1" customWidth="1"/>
@@ -13609,7 +13630,7 @@
       <c r="C236" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="D236" s="50" t="s">
+      <c r="D236" t="s">
         <v>1003</v>
       </c>
       <c r="E236" s="17">
@@ -13632,7 +13653,7 @@
       <c r="C237" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="D237" s="50" t="s">
+      <c r="D237" t="s">
         <v>1003</v>
       </c>
       <c r="E237" s="17">
@@ -13643,6 +13664,167 @@
       </c>
       <c r="G237" s="49" t="s">
         <v>1021</v>
+      </c>
+    </row>
+    <row r="238" spans="1:7" ht="30">
+      <c r="A238" s="20" t="s">
+        <v>87</v>
+      </c>
+      <c r="B238" s="20">
+        <v>400</v>
+      </c>
+      <c r="C238" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="D238" s="21" t="s">
+        <v>958</v>
+      </c>
+      <c r="E238" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="F238" s="27" t="s">
+        <v>858</v>
+      </c>
+      <c r="G238" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="239" spans="1:7">
+      <c r="A239" s="20" t="s">
+        <v>87</v>
+      </c>
+      <c r="B239" s="20">
+        <v>400</v>
+      </c>
+      <c r="C239" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="D239" s="21" t="s">
+        <v>958</v>
+      </c>
+      <c r="E239" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="F239" s="27" t="s">
+        <v>855</v>
+      </c>
+      <c r="G239" s="5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="240" spans="1:7">
+      <c r="A240" s="20" t="s">
+        <v>87</v>
+      </c>
+      <c r="B240" s="20">
+        <v>400</v>
+      </c>
+      <c r="C240" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="D240" s="21" t="s">
+        <v>958</v>
+      </c>
+      <c r="E240" s="27" t="s">
+        <v>23</v>
+      </c>
+      <c r="F240" s="27" t="s">
+        <v>856</v>
+      </c>
+      <c r="G240" s="5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="241" spans="1:7">
+      <c r="A241" s="20" t="s">
+        <v>87</v>
+      </c>
+      <c r="B241" s="20">
+        <v>400</v>
+      </c>
+      <c r="C241" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="D241" s="21" t="s">
+        <v>958</v>
+      </c>
+      <c r="E241" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="F241" s="27" t="s">
+        <v>857</v>
+      </c>
+      <c r="G241" s="5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="242" spans="1:7" ht="30">
+      <c r="A242" s="20" t="s">
+        <v>87</v>
+      </c>
+      <c r="B242" s="20">
+        <v>400</v>
+      </c>
+      <c r="C242" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="D242" s="21" t="s">
+        <v>958</v>
+      </c>
+      <c r="E242" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="F242" s="27" t="s">
+        <v>858</v>
+      </c>
+      <c r="G242" s="5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="243" spans="1:7" ht="30">
+      <c r="A243" s="20" t="s">
+        <v>87</v>
+      </c>
+      <c r="B243" s="20">
+        <v>400</v>
+      </c>
+      <c r="C243" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="D243" s="21" t="s">
+        <v>958</v>
+      </c>
+      <c r="E243" s="27" t="s">
+        <v>29</v>
+      </c>
+      <c r="F243" s="27" t="s">
+        <v>858</v>
+      </c>
+      <c r="G243" s="5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="244" spans="1:7" ht="30">
+      <c r="A244" s="20" t="s">
+        <v>87</v>
+      </c>
+      <c r="B244" s="20">
+        <v>400</v>
+      </c>
+      <c r="C244" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="D244" s="21" t="s">
+        <v>958</v>
+      </c>
+      <c r="E244" s="27" t="s">
+        <v>1044</v>
+      </c>
+      <c r="F244" s="27" t="s">
+        <v>858</v>
+      </c>
+      <c r="G244" s="5" t="s">
+        <v>1043</v>
       </c>
     </row>
   </sheetData>
@@ -20604,7 +20786,7 @@
       <c r="C19" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="D19" s="50" t="s">
+      <c r="D19" t="s">
         <v>970</v>
       </c>
       <c r="E19" s="24" t="s">
@@ -21078,19 +21260,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <TaxCatchAll xmlns="9cf85ca5-4acf-45da-adaa-d6bfc34b6c9f" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2595f96f-d2aa-4fa4-b5ed-10baae53ecb9">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100BD1EFD7F07544F4C8A5DF6ACE5557D0F" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="0a46465e297c47d8b88a71685f887e65">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="2595f96f-d2aa-4fa4-b5ed-10baae53ecb9" xmlns:ns3="9cf85ca5-4acf-45da-adaa-d6bfc34b6c9f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4503a5f252426d71f93d44927b16e869" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -21336,7 +21505,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -21345,25 +21514,20 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B3DC8D4E-C199-4BF9-AF5D-F16C7D7041E1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="2595f96f-d2aa-4fa4-b5ed-10baae53ecb9"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="9cf85ca5-4acf-45da-adaa-d6bfc34b6c9f"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <TaxCatchAll xmlns="9cf85ca5-4acf-45da-adaa-d6bfc34b6c9f" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2595f96f-d2aa-4fa4-b5ed-10baae53ecb9">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F11AB0D6-FBA0-4F11-8778-05A9ADBB93A5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -21383,10 +21547,28 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D590CCA9-7961-4660-BBC6-10104A0DDFD4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B3DC8D4E-C199-4BF9-AF5D-F16C7D7041E1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="2595f96f-d2aa-4fa4-b5ed-10baae53ecb9"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="9cf85ca5-4acf-45da-adaa-d6bfc34b6c9f"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>